<commit_message>
Add formatting to asset files (no data/structure changes)
Verified: row counts, column counts, and headers unchanged across all four files
(Ecommerce_Allocation_Request, Item_Code_allocation_table, Items_for_Replenishment,
Stores_Qtys_and_MinMax) - binary size changes are consistent with formatting only
(e.g. colors, borders, column widths).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Ecommerce_Allocation_Request.xlsx
+++ b/assets/Ecommerce_Allocation_Request.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9AD360F-966A-4597-BCBB-937307793D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="EcommerceAllocationRequest" state="visible" r:id="rId4"/>
+    <sheet name="EcommerceAllocationRequest" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -25,25 +29,39 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,12 +69,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -395,650 +446,654 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C58"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" style="1" customWidth="1"/>
+    <col min="2" max="3" width="9.7109375" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>470</v>
-      </c>
-      <c r="B2">
+      <c r="A2" s="3">
+        <v>470</v>
+      </c>
+      <c r="B2" s="4">
         <v>92425</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>470</v>
-      </c>
-      <c r="B3">
+      <c r="A3" s="3">
+        <v>470</v>
+      </c>
+      <c r="B3" s="4">
         <v>93306</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>470</v>
-      </c>
-      <c r="B4">
+      <c r="A4" s="3">
+        <v>470</v>
+      </c>
+      <c r="B4" s="4">
         <v>93307</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>470</v>
-      </c>
-      <c r="B5">
+      <c r="A5" s="3">
+        <v>470</v>
+      </c>
+      <c r="B5" s="4">
         <v>93329</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>470</v>
-      </c>
-      <c r="B6">
+      <c r="A6" s="3">
+        <v>470</v>
+      </c>
+      <c r="B6" s="4">
         <v>93332</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>470</v>
-      </c>
-      <c r="B7">
+      <c r="A7" s="3">
+        <v>470</v>
+      </c>
+      <c r="B7" s="4">
         <v>94916</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>470</v>
-      </c>
-      <c r="B8">
+      <c r="A8" s="3">
+        <v>470</v>
+      </c>
+      <c r="B8" s="4">
         <v>94917</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>470</v>
-      </c>
-      <c r="B9">
+      <c r="A9" s="3">
+        <v>470</v>
+      </c>
+      <c r="B9" s="4">
         <v>96933</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>470</v>
-      </c>
-      <c r="B10">
+      <c r="A10" s="3">
+        <v>470</v>
+      </c>
+      <c r="B10" s="4">
         <v>97526</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>470</v>
-      </c>
-      <c r="B11">
+      <c r="A11" s="3">
+        <v>470</v>
+      </c>
+      <c r="B11" s="4">
         <v>97527</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>470</v>
-      </c>
-      <c r="B12">
+      <c r="A12" s="3">
+        <v>470</v>
+      </c>
+      <c r="B12" s="4">
         <v>97528</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="4">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>470</v>
-      </c>
-      <c r="B13">
+      <c r="A13" s="3">
+        <v>470</v>
+      </c>
+      <c r="B13" s="4">
         <v>97668</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>470</v>
-      </c>
-      <c r="B14">
+      <c r="A14" s="3">
+        <v>470</v>
+      </c>
+      <c r="B14" s="4">
         <v>98412</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>470</v>
-      </c>
-      <c r="B15">
+      <c r="A15" s="3">
+        <v>470</v>
+      </c>
+      <c r="B15" s="4">
         <v>98413</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>470</v>
-      </c>
-      <c r="B16">
+      <c r="A16" s="3">
+        <v>470</v>
+      </c>
+      <c r="B16" s="4">
         <v>98414</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>470</v>
-      </c>
-      <c r="B17">
+      <c r="A17" s="3">
+        <v>470</v>
+      </c>
+      <c r="B17" s="4">
         <v>73723</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>470</v>
-      </c>
-      <c r="B18">
+      <c r="A18" s="3">
+        <v>470</v>
+      </c>
+      <c r="B18" s="4">
         <v>84852</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>470</v>
-      </c>
-      <c r="B19">
+      <c r="A19" s="3">
+        <v>470</v>
+      </c>
+      <c r="B19" s="4">
         <v>87418</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>470</v>
-      </c>
-      <c r="B20">
+      <c r="A20" s="3">
+        <v>470</v>
+      </c>
+      <c r="B20" s="4">
         <v>87419</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="4">
         <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>470</v>
-      </c>
-      <c r="B21">
+      <c r="A21" s="3">
+        <v>470</v>
+      </c>
+      <c r="B21" s="4">
         <v>87932</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>470</v>
-      </c>
-      <c r="B22">
+      <c r="A22" s="3">
+        <v>470</v>
+      </c>
+      <c r="B22" s="4">
         <v>87934</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>470</v>
-      </c>
-      <c r="B23">
+      <c r="A23" s="3">
+        <v>470</v>
+      </c>
+      <c r="B23" s="4">
         <v>87938</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="4">
         <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>470</v>
-      </c>
-      <c r="B24">
+      <c r="A24" s="3">
+        <v>470</v>
+      </c>
+      <c r="B24" s="4">
         <v>88656</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>470</v>
-      </c>
-      <c r="B25">
+      <c r="A25" s="3">
+        <v>470</v>
+      </c>
+      <c r="B25" s="4">
         <v>88657</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>470</v>
-      </c>
-      <c r="B26">
+      <c r="A26" s="3">
+        <v>470</v>
+      </c>
+      <c r="B26" s="4">
         <v>90922</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>470</v>
-      </c>
-      <c r="B27">
+      <c r="A27" s="3">
+        <v>470</v>
+      </c>
+      <c r="B27" s="4">
         <v>91208</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>470</v>
-      </c>
-      <c r="B28">
+      <c r="A28" s="3">
+        <v>470</v>
+      </c>
+      <c r="B28" s="4">
         <v>91209</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>470</v>
-      </c>
-      <c r="B29">
+      <c r="A29" s="3">
+        <v>470</v>
+      </c>
+      <c r="B29" s="4">
         <v>92409</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>470</v>
-      </c>
-      <c r="B30">
+      <c r="A30" s="3">
+        <v>470</v>
+      </c>
+      <c r="B30" s="4">
         <v>92413</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>470</v>
-      </c>
-      <c r="B31">
+      <c r="A31" s="3">
+        <v>470</v>
+      </c>
+      <c r="B31" s="4">
         <v>93240</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="4">
         <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>470</v>
-      </c>
-      <c r="B32">
+      <c r="A32" s="3">
+        <v>470</v>
+      </c>
+      <c r="B32" s="4">
         <v>94592</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="4">
         <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>470</v>
-      </c>
-      <c r="B33">
+      <c r="A33" s="3">
+        <v>470</v>
+      </c>
+      <c r="B33" s="4">
         <v>94593</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>470</v>
-      </c>
-      <c r="B34">
+      <c r="A34" s="3">
+        <v>470</v>
+      </c>
+      <c r="B34" s="4">
         <v>94594</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>470</v>
-      </c>
-      <c r="B35">
+      <c r="A35" s="3">
+        <v>470</v>
+      </c>
+      <c r="B35" s="4">
         <v>94595</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>470</v>
-      </c>
-      <c r="B36">
+      <c r="A36" s="3">
+        <v>470</v>
+      </c>
+      <c r="B36" s="4">
         <v>97346</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>470</v>
-      </c>
-      <c r="B37">
+      <c r="A37" s="3">
+        <v>470</v>
+      </c>
+      <c r="B37" s="4">
         <v>97352</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>470</v>
-      </c>
-      <c r="B38">
+      <c r="A38" s="3">
+        <v>470</v>
+      </c>
+      <c r="B38" s="4">
         <v>97360</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>470</v>
-      </c>
-      <c r="B39">
+      <c r="A39" s="3">
+        <v>470</v>
+      </c>
+      <c r="B39" s="4">
         <v>97449</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>470</v>
-      </c>
-      <c r="B40">
+      <c r="A40" s="3">
+        <v>470</v>
+      </c>
+      <c r="B40" s="4">
         <v>98495</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>470</v>
-      </c>
-      <c r="B41">
+      <c r="A41" s="3">
+        <v>470</v>
+      </c>
+      <c r="B41" s="4">
         <v>69378</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>470</v>
-      </c>
-      <c r="B42">
+      <c r="A42" s="3">
+        <v>470</v>
+      </c>
+      <c r="B42" s="4">
         <v>69382</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>470</v>
-      </c>
-      <c r="B43">
+      <c r="A43" s="3">
+        <v>470</v>
+      </c>
+      <c r="B43" s="4">
         <v>69389</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>470</v>
-      </c>
-      <c r="B44">
+      <c r="A44" s="3">
+        <v>470</v>
+      </c>
+      <c r="B44" s="4">
         <v>92767</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>470</v>
-      </c>
-      <c r="B45">
+      <c r="A45" s="3">
+        <v>470</v>
+      </c>
+      <c r="B45" s="4">
         <v>97558</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>470</v>
-      </c>
-      <c r="B46">
+      <c r="A46" s="3">
+        <v>470</v>
+      </c>
+      <c r="B46" s="4">
         <v>97567</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>470</v>
-      </c>
-      <c r="B47">
+      <c r="A47" s="3">
+        <v>470</v>
+      </c>
+      <c r="B47" s="4">
         <v>97580</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>470</v>
-      </c>
-      <c r="B48">
+      <c r="A48" s="3">
+        <v>470</v>
+      </c>
+      <c r="B48" s="4">
         <v>97605</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>470</v>
-      </c>
-      <c r="B49">
+      <c r="A49" s="3">
+        <v>470</v>
+      </c>
+      <c r="B49" s="4">
         <v>97665</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="4">
         <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>470</v>
-      </c>
-      <c r="B50">
+      <c r="A50" s="3">
+        <v>470</v>
+      </c>
+      <c r="B50" s="4">
         <v>75924</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>470</v>
-      </c>
-      <c r="B51">
+      <c r="A51" s="3">
+        <v>470</v>
+      </c>
+      <c r="B51" s="4">
         <v>80679</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>470</v>
-      </c>
-      <c r="B52">
+      <c r="A52" s="3">
+        <v>470</v>
+      </c>
+      <c r="B52" s="4">
         <v>83163</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="4">
         <v>24</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>470</v>
-      </c>
-      <c r="B53">
+      <c r="A53" s="3">
+        <v>470</v>
+      </c>
+      <c r="B53" s="4">
         <v>84802</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>470</v>
-      </c>
-      <c r="B54">
+      <c r="A54" s="3">
+        <v>470</v>
+      </c>
+      <c r="B54" s="4">
         <v>87635</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>470</v>
-      </c>
-      <c r="B55">
+      <c r="A55" s="3">
+        <v>470</v>
+      </c>
+      <c r="B55" s="4">
         <v>91653</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>470</v>
-      </c>
-      <c r="B56">
+      <c r="A56" s="3">
+        <v>470</v>
+      </c>
+      <c r="B56" s="4">
         <v>97067</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="4">
         <v>24</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>470</v>
-      </c>
-      <c r="B57">
+      <c r="A57" s="3">
+        <v>470</v>
+      </c>
+      <c r="B57" s="4">
         <v>98152</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>470</v>
-      </c>
-      <c r="B58">
+      <c r="A58" s="3">
+        <v>470</v>
+      </c>
+      <c r="B58" s="4">
         <v>98177</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="4">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>